<commit_message>
add excel QA risk catalog
</commit_message>
<xml_diff>
--- a/phon_book/docs/QA_RISK_CATALOG.xlsx
+++ b/phon_book/docs/QA_RISK_CATALOG.xlsx
@@ -416,21 +416,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,6 +497,21 @@
           <t>Notes / Ambiguity</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Validation Status</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Validation Evidence</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Validation Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -556,6 +574,21 @@
           <t>none</t>
         </is>
       </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>Signing in with email placed in the username field returned a plain string error and crashed the server. Reply: User amir@example.com does not exist.</t>
+        </is>
+      </c>
+      <c r="O2" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -618,6 +651,21 @@
           <t>none</t>
         </is>
       </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>After one signup initialized the schema, add_phone_user and get_all_phone_users both succeeded without any sign_in step.</t>
+        </is>
+      </c>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -680,6 +728,21 @@
           <t>ownership is not explicitly modeled in the schema and should be treated as a major mismatch risk</t>
         </is>
       </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
+          <t>Code-confirmed / runtime not directly isolated</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="inlineStr">
+        <is>
+          <t>Schema and handlers still show no ownership relation between auth users and phonebook contacts. Multi-user isolation was not directly executed in this pass.</t>
+        </is>
+      </c>
+      <c r="O4" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -742,6 +805,21 @@
           <t>none</t>
         </is>
       </c>
+      <c r="M5" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N5" s="1" t="inlineStr">
+        <is>
+          <t>Two different usernames were registered successfully with the same email in one batch.</t>
+        </is>
+      </c>
+      <c r="O5" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -804,6 +882,21 @@
           <t>the assignment does not specify strict regex-style validation, so the exact acceptance rule may need to be framed as expected validation quality rather than a hard requirement</t>
         </is>
       </c>
+      <c r="M6" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N6" s="1" t="inlineStr">
+        <is>
+          <t>Signup with email value abc succeeded.</t>
+        </is>
+      </c>
+      <c r="O6" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -866,6 +959,21 @@
           <t>same pattern likely affects multiple commands beyond auth</t>
         </is>
       </c>
+      <c r="M7" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="inlineStr">
+        <is>
+          <t>Signup missing username returned plain string KeyError and terminated the server.</t>
+        </is>
+      </c>
+      <c r="O7" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -928,6 +1036,21 @@
           <t>similar integrity-failure behavior may occur for other unique fields</t>
         </is>
       </c>
+      <c r="M8" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N8" s="1" t="inlineStr">
+        <is>
+          <t>Duplicate username signup replied with raw UNIQUE constraint failed and terminated the server.</t>
+        </is>
+      </c>
+      <c r="O8" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -990,6 +1113,21 @@
           <t>exact crash behavior may vary by field and command</t>
         </is>
       </c>
+      <c r="M9" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N9" s="1" t="inlineStr">
+        <is>
+          <t>Signup with integer password returned plain string AttributeError and terminated the server.</t>
+        </is>
+      </c>
+      <c r="O9" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1052,6 +1190,21 @@
           <t>exact exploitability depends on how commands are submitted in practice, but the state model is weak</t>
         </is>
       </c>
+      <c r="M10" s="1" t="inlineStr">
+        <is>
+          <t>Code-confirmed / runtime not isolated</t>
+        </is>
+      </c>
+      <c r="N10" s="1" t="inlineStr">
+        <is>
+          <t>Logout logic removes any provided username from online_users without request ownership checks. Not directly isolated through protocol in this pass.</t>
+        </is>
+      </c>
+      <c r="O10" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1114,6 +1267,21 @@
           <t>contract behavior should be verified separately for business errors and unexpected exceptions</t>
         </is>
       </c>
+      <c r="M11" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N11" s="1" t="inlineStr">
+        <is>
+          <t>Failure replies were plain strings such as KeyError text and UNIQUE constraint text instead of structured command_name/result objects.</t>
+        </is>
+      </c>
+      <c r="O11" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1176,6 +1344,21 @@
           <t>closely related to error-handling risks but retained here because of its direct operational impact</t>
         </is>
       </c>
+      <c r="M12" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N12" s="1" t="inlineStr">
+        <is>
+          <t>Several invalid requests terminated the server and required a restart for the next test.</t>
+        </is>
+      </c>
+      <c r="O12" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1238,6 +1421,21 @@
           <t>whether partial success is acceptable is not explicitly defined by the assignment</t>
         </is>
       </c>
+      <c r="M13" s="1" t="inlineStr">
+        <is>
+          <t>Not yet validated</t>
+        </is>
+      </c>
+      <c r="N13" s="1" t="inlineStr">
+        <is>
+          <t>Batch partial-success behavior was inferred from code only in this pass.</t>
+        </is>
+      </c>
+      <c r="O13" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -1300,6 +1498,21 @@
           <t>this is expected DB behavior technically, but it is still a QA risk if not managed</t>
         </is>
       </c>
+      <c r="M14" s="1" t="inlineStr">
+        <is>
+          <t>Known operational condition</t>
+        </is>
+      </c>
+      <c r="N14" s="1" t="inlineStr">
+        <is>
+          <t>Existing persistent sab.db was present in the working copy, so tests were moved to a temporary isolated copy to avoid contamination.</t>
+        </is>
+      </c>
+      <c r="O14" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1362,6 +1575,21 @@
           <t>exact runtime behavior should be verified for both create and edit paths</t>
         </is>
       </c>
+      <c r="M15" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N15" s="1" t="inlineStr">
+        <is>
+          <t>Duplicate contact name and duplicate phone number both returned raw UNIQUE constraint errors and terminated the server.</t>
+        </is>
+      </c>
+      <c r="O15" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -1424,6 +1652,21 @@
           <t>some commands may fail with key errors while others fail later at the ORM layer</t>
         </is>
       </c>
+      <c r="M16" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N16" s="1" t="inlineStr">
+        <is>
+          <t>add_phone_user missing phone_number returned plain string KeyError and terminated the server.</t>
+        </is>
+      </c>
+      <c r="O16" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -1486,6 +1729,21 @@
           <t>delete may behave differently from get/edit because delete uses a query execution path rather than .get(...)</t>
         </is>
       </c>
+      <c r="M17" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N17" s="1" t="inlineStr">
+        <is>
+          <t>add_phone_number for a non-existing contact returned raw PhoneUsersDoesNotExist details and terminated the server after schema initialization.</t>
+        </is>
+      </c>
+      <c r="O17" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -1548,6 +1806,21 @@
           <t>the exact exposure level depends on the triggering exception type</t>
         </is>
       </c>
+      <c r="M18" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N18" s="1" t="inlineStr">
+        <is>
+          <t>Server output exposed full tracebacks and replies exposed internal exception text and SQL details.</t>
+        </is>
+      </c>
+      <c r="O18" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -1610,6 +1883,21 @@
           <t>this is a security-hardening concern rather than a direct functional defect</t>
         </is>
       </c>
+      <c r="M19" s="1" t="inlineStr">
+        <is>
+          <t>Code-confirmed</t>
+        </is>
+      </c>
+      <c r="N19" s="1" t="inlineStr">
+        <is>
+          <t>bcrypt is used with a low rounds value in code inspection. Runtime functional validation is not applicable.</t>
+        </is>
+      </c>
+      <c r="O19" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -1672,6 +1960,21 @@
           <t>actual concurrency behavior depends on runtime request scheduling and the chosen execution model</t>
         </is>
       </c>
+      <c r="M20" s="1" t="inlineStr">
+        <is>
+          <t>Not yet validated</t>
+        </is>
+      </c>
+      <c r="N20" s="1" t="inlineStr">
+        <is>
+          <t>Concurrent behavior was not executed in this validation pass.</t>
+        </is>
+      </c>
+      <c r="O20" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1732,6 +2035,98 @@
       <c r="L21" s="1" t="inlineStr">
         <is>
           <t>exact manifestation depends on runtime concurrency and DB locking behavior</t>
+        </is>
+      </c>
+      <c r="M21" s="1" t="inlineStr">
+        <is>
+          <t>Not yet validated</t>
+        </is>
+      </c>
+      <c r="N21" s="1" t="inlineStr">
+        <is>
+          <t>Concurrent duplicate creation was not executed in this validation pass.</t>
+        </is>
+      </c>
+      <c r="O21" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>RISK-021</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Phonebook tables are not initialized before the first phonebook operation</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>Persistence and Data Consistency Risks</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>If a phonebook command is the first database-touching operation after startup, the required phonebook tables may not exist and the server can fail with a raw OperationalError.</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>The system should support contact-management commands without depending on a prior auth command for schema creation.</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>Running add_phone_user or add_phone_number as the first operation on a clean database returned no such table: phone_user_table and terminated the server. The table-creation path currently depends on auth-side before_request usage.</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>Valid phonebook operations can fail purely due to command ordering, and the server can terminate on first contact-management use.</t>
+        </is>
+      </c>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J22" s="1" t="inlineStr">
+        <is>
+          <t>manual runtime test; code inspection; schema initialization behavior</t>
+        </is>
+      </c>
+      <c r="K22" s="1" t="inlineStr">
+        <is>
+          <t>manual startup-path test; automated integration test covering first phonebook operation on clean DB</t>
+        </is>
+      </c>
+      <c r="L22" s="1" t="inlineStr">
+        <is>
+          <t>This is distinct from general authorization risk because it happens before business-rule evaluation and depends on schema initialization order.</t>
+        </is>
+      </c>
+      <c r="M22" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="N22" s="1" t="inlineStr">
+        <is>
+          <t>On a clean database, add_phone_user and add_phone_number both failed with no such table: phone_user_table until signup had run first.</t>
+        </is>
+      </c>
+      <c r="O22" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>

</xml_diff>